<commit_message>
feat: update Alíquota.xlsx with new data
</commit_message>
<xml_diff>
--- a/botCTE/botCTE/Alíquota.xlsx
+++ b/botCTE/botCTE/Alíquota.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Artur Senna\PycharmProjects\botCityCTE\botCTE\botCTE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brian Marques\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA060CC-117A-4F19-AC2B-2CFECD5F5B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{078037D6-CD6C-4CFD-9F08-81BA3DBE324A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA807991-941E-477F-BBBF-867C6D8017B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,6 +37,9 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="28">
+  <si>
+    <t>UF</t>
+  </si>
   <si>
     <t>AC</t>
   </si>
@@ -68,13 +71,13 @@
     <t>MA</t>
   </si>
   <si>
-    <t>MG</t>
+    <t>MT</t>
   </si>
   <si>
     <t>MS</t>
   </si>
   <si>
-    <t>MT</t>
+    <t>MG</t>
   </si>
   <si>
     <t>PA</t>
@@ -83,19 +86,19 @@
     <t>PB</t>
   </si>
   <si>
+    <t>PR</t>
+  </si>
+  <si>
     <t>PE</t>
   </si>
   <si>
     <t>PI</t>
   </si>
   <si>
-    <t>PR</t>
+    <t>RN</t>
   </si>
   <si>
     <t>RJ</t>
-  </si>
-  <si>
-    <t>RN</t>
   </si>
   <si>
     <t>RO</t>
@@ -110,16 +113,13 @@
     <t>SC</t>
   </si>
   <si>
+    <t>SP</t>
+  </si>
+  <si>
     <t>SE</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
     <t>TO</t>
-  </si>
-  <si>
-    <t>UF</t>
   </si>
 </sst>
 </file>
@@ -129,7 +129,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -397,9 +397,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -437,7 +437,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -543,7 +543,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -685,7 +685,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -694,103 +694,103 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6596CEC0-C1AD-42F0-9A7D-CB3E5481D5E4}">
   <dimension ref="A1:AC28"/>
-  <sheetFormatPr defaultColWidth="4.140625" defaultRowHeight="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="4.140625" defaultRowHeight="17.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4.140625" style="17"/>
     <col min="2" max="28" width="5.5703125" style="18" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="4.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="1" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" s="1" customFormat="1" ht="17.25" customHeight="1" thickBot="1">
       <c r="A1" s="4" t="s">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="S1" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T1" s="6" t="s">
         <v>19</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y1" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z1" s="6" t="s">
         <v>25</v>
       </c>
       <c r="AA1" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="AB1" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AC1" s="2"/>
     </row>
-    <row r="2" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" ht="17.25" customHeight="1">
       <c r="A2" s="7" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="8">
         <v>19</v>
@@ -874,15 +874,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" ht="17.25" customHeight="1">
       <c r="A3" s="7" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="11">
         <v>12</v>
       </c>
       <c r="C3" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" s="12">
         <v>12</v>
@@ -960,9 +960,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" ht="17.25" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="11">
         <v>12</v>
@@ -971,7 +971,7 @@
         <v>12</v>
       </c>
       <c r="D4" s="5">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E4" s="12">
         <v>12</v>
@@ -1046,9 +1046,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" ht="17.25" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="11">
         <v>12</v>
@@ -1132,9 +1132,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" ht="17.25" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="11">
         <v>12</v>
@@ -1149,7 +1149,7 @@
         <v>12</v>
       </c>
       <c r="F6" s="5">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="G6" s="12">
         <v>12</v>
@@ -1218,9 +1218,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" ht="17.25" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" s="11">
         <v>12</v>
@@ -1304,9 +1304,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" ht="17.25" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" s="11">
         <v>12</v>
@@ -1327,7 +1327,7 @@
         <v>12</v>
       </c>
       <c r="H8" s="5">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I8" s="12">
         <v>12</v>
@@ -1390,95 +1390,95 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" ht="17.25" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" s="11">
-        <v>7</v>
-      </c>
-      <c r="C9" s="12">
-        <v>7</v>
-      </c>
-      <c r="D9" s="12">
-        <v>7</v>
-      </c>
-      <c r="E9" s="12">
-        <v>7</v>
-      </c>
-      <c r="F9" s="12">
-        <v>7</v>
-      </c>
-      <c r="G9" s="12">
-        <v>7</v>
-      </c>
-      <c r="H9" s="12">
-        <v>7</v>
+        <v>12</v>
+      </c>
+      <c r="C9" s="11">
+        <v>12</v>
+      </c>
+      <c r="D9" s="11">
+        <v>12</v>
+      </c>
+      <c r="E9" s="11">
+        <v>12</v>
+      </c>
+      <c r="F9" s="11">
+        <v>12</v>
+      </c>
+      <c r="G9" s="11">
+        <v>12</v>
+      </c>
+      <c r="H9" s="11">
+        <v>12</v>
       </c>
       <c r="I9" s="5">
         <v>17</v>
       </c>
-      <c r="J9" s="12">
-        <v>7</v>
-      </c>
-      <c r="K9" s="12">
-        <v>7</v>
-      </c>
-      <c r="L9" s="12">
-        <v>7</v>
-      </c>
-      <c r="M9" s="12">
-        <v>7</v>
-      </c>
-      <c r="N9" s="12">
-        <v>12</v>
-      </c>
-      <c r="O9" s="12">
-        <v>7</v>
-      </c>
-      <c r="P9" s="12">
-        <v>7</v>
-      </c>
-      <c r="Q9" s="12">
-        <v>12</v>
-      </c>
-      <c r="R9" s="12">
-        <v>7</v>
-      </c>
-      <c r="S9" s="12">
-        <v>7</v>
-      </c>
-      <c r="T9" s="12">
-        <v>7</v>
-      </c>
-      <c r="U9" s="12">
-        <v>12</v>
-      </c>
-      <c r="V9" s="12">
-        <v>7</v>
-      </c>
-      <c r="W9" s="12">
-        <v>7</v>
-      </c>
-      <c r="X9" s="12">
-        <v>12</v>
-      </c>
-      <c r="Y9" s="12">
-        <v>12</v>
-      </c>
-      <c r="Z9" s="12">
-        <v>12</v>
-      </c>
-      <c r="AA9" s="12">
-        <v>7</v>
-      </c>
-      <c r="AB9" s="13">
-        <v>7</v>
+      <c r="J9" s="11">
+        <v>12</v>
+      </c>
+      <c r="K9" s="11">
+        <v>12</v>
+      </c>
+      <c r="L9" s="11">
+        <v>12</v>
+      </c>
+      <c r="M9" s="11">
+        <v>12</v>
+      </c>
+      <c r="N9" s="11">
+        <v>12</v>
+      </c>
+      <c r="O9" s="11">
+        <v>12</v>
+      </c>
+      <c r="P9" s="11">
+        <v>12</v>
+      </c>
+      <c r="Q9" s="11">
+        <v>12</v>
+      </c>
+      <c r="R9" s="11">
+        <v>12</v>
+      </c>
+      <c r="S9" s="11">
+        <v>12</v>
+      </c>
+      <c r="T9" s="11">
+        <v>12</v>
+      </c>
+      <c r="U9" s="11">
+        <v>12</v>
+      </c>
+      <c r="V9" s="11">
+        <v>12</v>
+      </c>
+      <c r="W9" s="11">
+        <v>12</v>
+      </c>
+      <c r="X9" s="11">
+        <v>12</v>
+      </c>
+      <c r="Y9" s="11">
+        <v>12</v>
+      </c>
+      <c r="Z9" s="11">
+        <v>12</v>
+      </c>
+      <c r="AA9" s="11">
+        <v>12</v>
+      </c>
+      <c r="AB9" s="11">
+        <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" ht="17.25" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" s="11">
         <v>12</v>
@@ -1562,9 +1562,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="17.25" customHeight="1">
       <c r="A11" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" s="11">
         <v>12</v>
@@ -1648,9 +1648,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" ht="17.25" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="11">
         <v>12</v>
@@ -1734,9 +1734,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="17.25" customHeight="1">
       <c r="A13" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" s="11">
         <v>12</v>
@@ -1820,9 +1820,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" ht="17.25" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B14" s="11">
         <v>7</v>
@@ -1846,7 +1846,7 @@
         <v>7</v>
       </c>
       <c r="I14" s="12">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J14" s="12">
         <v>7</v>
@@ -1906,9 +1906,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" ht="17.25" customHeight="1">
       <c r="A15" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" s="11">
         <v>12</v>
@@ -1992,9 +1992,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" ht="17.25" customHeight="1">
       <c r="A16" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" s="11">
         <v>12</v>
@@ -2078,95 +2078,95 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" ht="17.25" customHeight="1">
       <c r="A17" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11">
+        <v>7</v>
+      </c>
+      <c r="C17" s="12">
+        <v>7</v>
+      </c>
+      <c r="D17" s="12">
+        <v>7</v>
+      </c>
+      <c r="E17" s="12">
+        <v>7</v>
+      </c>
+      <c r="F17" s="12">
+        <v>7</v>
+      </c>
+      <c r="G17" s="12">
+        <v>7</v>
+      </c>
+      <c r="H17" s="12">
+        <v>7</v>
+      </c>
+      <c r="I17" s="12">
+        <v>7</v>
+      </c>
+      <c r="J17" s="12">
+        <v>7</v>
+      </c>
+      <c r="K17" s="12">
+        <v>7</v>
+      </c>
+      <c r="L17" s="12">
+        <v>7</v>
+      </c>
+      <c r="M17" s="12">
+        <v>7</v>
+      </c>
+      <c r="N17" s="12">
+        <v>12</v>
+      </c>
+      <c r="O17" s="12">
+        <v>7</v>
+      </c>
+      <c r="P17" s="12">
+        <v>7</v>
+      </c>
+      <c r="Q17" s="5">
+        <v>19.5</v>
+      </c>
+      <c r="R17" s="12">
+        <v>7</v>
+      </c>
+      <c r="S17" s="12">
+        <v>7</v>
+      </c>
+      <c r="T17" s="12">
+        <v>7</v>
+      </c>
+      <c r="U17" s="12">
+        <v>12</v>
+      </c>
+      <c r="V17" s="12">
+        <v>7</v>
+      </c>
+      <c r="W17" s="12">
+        <v>7</v>
+      </c>
+      <c r="X17" s="12">
+        <v>12</v>
+      </c>
+      <c r="Y17" s="12">
+        <v>12</v>
+      </c>
+      <c r="Z17" s="12">
+        <v>12</v>
+      </c>
+      <c r="AA17" s="12">
+        <v>7</v>
+      </c>
+      <c r="AB17" s="13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" ht="17.25" customHeight="1">
+      <c r="A18" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="B17" s="11">
-        <v>7</v>
-      </c>
-      <c r="C17" s="12">
-        <v>7</v>
-      </c>
-      <c r="D17" s="12">
-        <v>7</v>
-      </c>
-      <c r="E17" s="12">
-        <v>7</v>
-      </c>
-      <c r="F17" s="12">
-        <v>7</v>
-      </c>
-      <c r="G17" s="12">
-        <v>7</v>
-      </c>
-      <c r="H17" s="12">
-        <v>7</v>
-      </c>
-      <c r="I17" s="12">
-        <v>12</v>
-      </c>
-      <c r="J17" s="12">
-        <v>7</v>
-      </c>
-      <c r="K17" s="12">
-        <v>7</v>
-      </c>
-      <c r="L17" s="12">
-        <v>7</v>
-      </c>
-      <c r="M17" s="12">
-        <v>7</v>
-      </c>
-      <c r="N17" s="12">
-        <v>12</v>
-      </c>
-      <c r="O17" s="12">
-        <v>7</v>
-      </c>
-      <c r="P17" s="12">
-        <v>7</v>
-      </c>
-      <c r="Q17" s="5">
-        <v>19</v>
-      </c>
-      <c r="R17" s="12">
-        <v>7</v>
-      </c>
-      <c r="S17" s="12">
-        <v>7</v>
-      </c>
-      <c r="T17" s="12">
-        <v>7</v>
-      </c>
-      <c r="U17" s="12">
-        <v>12</v>
-      </c>
-      <c r="V17" s="12">
-        <v>7</v>
-      </c>
-      <c r="W17" s="12">
-        <v>7</v>
-      </c>
-      <c r="X17" s="12">
-        <v>12</v>
-      </c>
-      <c r="Y17" s="12">
-        <v>12</v>
-      </c>
-      <c r="Z17" s="12">
-        <v>12</v>
-      </c>
-      <c r="AA17" s="12">
-        <v>7</v>
-      </c>
-      <c r="AB17" s="13">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>15</v>
       </c>
       <c r="B18" s="11">
         <v>12</v>
@@ -2250,9 +2250,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" ht="17.25" customHeight="1">
       <c r="A19" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B19" s="11">
         <v>12</v>
@@ -2336,7 +2336,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" ht="17.25" customHeight="1">
       <c r="A20" s="7" t="s">
         <v>19</v>
       </c>
@@ -2422,9 +2422,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" ht="17.25" customHeight="1">
       <c r="A21" s="7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B21" s="11">
         <v>7</v>
@@ -2448,7 +2448,7 @@
         <v>7</v>
       </c>
       <c r="I21" s="12">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J21" s="12">
         <v>7</v>
@@ -2484,7 +2484,7 @@
         <v>7</v>
       </c>
       <c r="U21" s="5">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="V21" s="12">
         <v>7</v>
@@ -2508,9 +2508,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" ht="17.25" customHeight="1">
       <c r="A22" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22" s="11">
         <v>12</v>
@@ -2594,9 +2594,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" ht="17.25" customHeight="1">
       <c r="A23" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23" s="11">
         <v>12</v>
@@ -2680,9 +2680,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" ht="17.25" customHeight="1">
       <c r="A24" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" s="11">
         <v>7</v>
@@ -2706,7 +2706,7 @@
         <v>7</v>
       </c>
       <c r="I24" s="12">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J24" s="12">
         <v>7</v>
@@ -2751,7 +2751,7 @@
         <v>7</v>
       </c>
       <c r="X24" s="5">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="Y24" s="12">
         <v>12</v>
@@ -2766,9 +2766,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" ht="17.25" customHeight="1">
       <c r="A25" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" s="11">
         <v>7</v>
@@ -2792,7 +2792,7 @@
         <v>7</v>
       </c>
       <c r="I25" s="12">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J25" s="12">
         <v>7</v>
@@ -2852,7 +2852,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" ht="17.25" customHeight="1">
       <c r="A26" s="7" t="s">
         <v>25</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>7</v>
       </c>
       <c r="I26" s="12">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J26" s="12">
         <v>7</v>
@@ -2932,15 +2932,15 @@
         <v>18</v>
       </c>
       <c r="AA26" s="12">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="AB26" s="13">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" ht="17.25" customHeight="1">
       <c r="A27" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B27" s="11">
         <v>12</v>
@@ -3018,15 +3018,15 @@
         <v>12</v>
       </c>
       <c r="AA27" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AB27" s="13">
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:28" ht="17.25" customHeight="1" thickBot="1">
       <c r="A28" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" s="14">
         <v>12</v>

</xml_diff>